<commit_message>
Web interface into AI studio
modular configurations and test environments
</commit_message>
<xml_diff>
--- a/notebook/dataset/Triage-Module-Evaluation-Checkpoint.xlsx
+++ b/notebook/dataset/Triage-Module-Evaluation-Checkpoint.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,36 +425,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>prompts</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>language</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>llm_normalized_output</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>llm_detected_language</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Detected Language</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Normalized Output</t>
         </is>
@@ -468,7 +480,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The employer holds the passport of the employee, is this legal?</t>
+          <t>&lt;The employer holds the passport of the employee. Is this legal?&gt;</t>
         </is>
       </c>
     </row>
@@ -492,7 +504,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>I was not permitted to take a 3-month leave by my employer.</t>
+          <t>&lt;It is alleged that the employee was not allowed to take a 3-month leave from the employer.&gt;</t>
         </is>
       </c>
     </row>
@@ -516,7 +528,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Can I file a complaint if my pet is harming me?</t>
+          <t>&lt;Does the owner have the right to file a complaint if they are being harmed by their pet?&gt;</t>
         </is>
       </c>
     </row>
@@ -540,7 +552,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>I wish to return home but the ticket is not being given to me.</t>
+          <t>&lt;It is alleged that the person wants to go home but the ticket is not being given to them.&gt;</t>
         </is>
       </c>
     </row>
@@ -564,7 +576,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>I was presented with a contract different from what was discussed with the agency.</t>
+          <t>&lt;It is alleged that the contract I signed is different from what was discussed with the agency.&gt;</t>
         </is>
       </c>
     </row>
@@ -588,7 +600,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>What is the legal basis for deducting my salary for meals?</t>
+          <t>&lt;It is alleged that the salary is being withheld for food purposes.&gt;</t>
         </is>
       </c>
     </row>
@@ -612,7 +624,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>I did not receive any separation pay when I was terminated.</t>
+          <t>&lt;Wala po akong natanggap na separation pay nung tinanggal ako.&gt;</t>
         </is>
       </c>
     </row>
@@ -636,7 +648,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>How to file a complaint with DOLE while abroad</t>
+          <t>&lt;How to file a complaint with DOLE if you are abroad&gt;</t>
         </is>
       </c>
     </row>
@@ -660,7 +672,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Can an employer detain an employee if they flee?</t>
+          <t>&lt;Pwede ba akong ipakulong ng amo ko kung tatakas ako?&gt;</t>
         </is>
       </c>
     </row>
@@ -684,7 +696,8 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>The employer did not pay SSS and PhilHealth contributions despite being required to do so.</t>
+          <t>&lt;Normalized English Text&gt;
+It is alleged that the employer does not pay SSS and PhilHealth contributions despite being required to do so.</t>
         </is>
       </c>
     </row>
@@ -701,16 +714,8 @@
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>The contract has been completed but the party is refusing to allow the employee to return.</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -725,16 +730,8 @@
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>I work more than 16 hours per day, is this prohibited?</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -749,16 +746,8 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>The agency took my cellphone, it is forbidden to communicate with family.</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -773,16 +762,8 @@
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Can an employee switch employers before the contract is completed?</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -797,16 +778,8 @@
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>What should be done if the individual is blacklisted by immigration?</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -821,16 +794,8 @@
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Would I be subject to penalties for not complying with the minimum wage?</t>
-        </is>
-      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -845,16 +810,8 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Terminated for alleged theft.</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -869,16 +826,8 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Is it legal to reduce my salary if I damage company property?</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -893,16 +842,8 @@
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>I am being forced to sleep on the kitchen floor, can this be reported?</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -917,16 +858,8 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Delayed salary for two months, what are my rights?</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -941,16 +874,8 @@
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>The employer refuses to sign my release paper.</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -965,16 +890,8 @@
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>I am pregnant and they want to send me back, is that legal?</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -989,16 +906,8 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Paid the agency fee again for renewal.</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1013,16 +922,8 @@
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>I am ill but refuse to be taken to the hospital.</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1037,16 +938,8 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Can a person apply for a visa while having debts with a lender?</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1061,16 +954,8 @@
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>The employer is hiding the employment contract.</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1085,16 +970,8 @@
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>I was forced to work at the employer's other house.</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1109,16 +986,8 @@
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>What is the penalty for illegal recruitment?</t>
-        </is>
-      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1133,16 +1002,8 @@
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Does the contract include free food and accommodation?</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1157,16 +1018,8 @@
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Can a domestic helper demand overtime pay?</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1181,16 +1034,8 @@
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>I am being harassed by my employer's spouse.</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1205,16 +1050,8 @@
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>I wish to recover the placement fee paid.</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1229,16 +1066,8 @@
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>I am afraid to report because I might be deported.</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1253,16 +1082,8 @@
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Is the visa still valid if the employee was terminated yesterday?</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1277,16 +1098,8 @@
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>What is required for an OEC when returning briefly?</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1301,16 +1114,8 @@
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Who will pay for my plane ticket home?</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1325,16 +1130,8 @@
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Can a case be filed with POEA online?</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1349,16 +1146,8 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>The former employer refuses to provide a reference letter.</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1373,16 +1162,8 @@
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Moved to night shift without prior notice.</t>
-        </is>
-      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1397,16 +1178,8 @@
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>I was prohibited from leaving during my day off.</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1421,16 +1194,8 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Can an employee take a part-time job during days off?</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1445,16 +1210,8 @@
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>What should be done if my passport is lost?</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1469,16 +1226,8 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Sent money to the agency but it was a scam.</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1493,16 +1242,8 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>I am being harassed by a lending collector in the Philippines.</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1517,16 +1258,8 @@
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Can a breach of contract lawsuit be filed in the Philippines?</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1541,16 +1274,8 @@
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Should the embassy have the right to send me back?</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1565,16 +1290,8 @@
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>I did not receive the last payment before leaving.</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1589,16 +1306,8 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>I am being charged for the damaged washing machine.</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1613,16 +1322,8 @@
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>The employer is always late in paying wages.</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1637,16 +1338,8 @@
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>I would like to know the status of my case at the NLRC.</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1661,16 +1354,8 @@
       </c>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Termination is valid if communicated through text message only?</t>
-        </is>
-      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1685,16 +1370,8 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>I overstayed by 2 days, will this cause problems with Immigration?</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1709,16 +1386,8 @@
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Employee's employer refuses to provide separation pay, what to do?</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1733,16 +1402,8 @@
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Check if the agency being spoken to is legitimate.</t>
-        </is>
-      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1757,16 +1418,8 @@
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Must an OFW pay tax in the Philippines?</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1781,16 +1434,8 @@
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Help, I am being verbally harassed by my employer, can I file a complaint?</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1805,16 +1450,8 @@
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Please advise, the party wishes to terminate the contract because of toxic conditions.</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1829,16 +1466,8 @@
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>No food allowance provided, is that legal?</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1853,16 +1482,8 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>The employer confiscated the employee's phone. Is this permissible?</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1877,16 +1498,8 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Can a case be filed directly with the Hong Kong Labour Department?</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1901,16 +1514,8 @@
       </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>How to claim Long Service Payment after 5 years?</t>
-        </is>
-      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1925,16 +1530,8 @@
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>I lost my passport, how can I return home?</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1949,16 +1546,8 @@
       </c>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Need a medical certificate when renewing a contract?</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1973,16 +1562,8 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>The agency I am associated with is requesting an additional fee, is this a scam?</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1997,16 +1578,8 @@
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Is it legal to reduce my salary due to the pandemic?</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2021,16 +1594,8 @@
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Taglish</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Can an employee transfer to another employer after being terminated?</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2045,16 +1610,8 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>I was denied the return plane ticket, what are my rights?</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2069,16 +1626,8 @@
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>I have a pending case in the Philippines, is it possible to leave?</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2093,16 +1642,8 @@
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Taglish</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>I was required to work on Sundays, which is not allowed.</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2117,16 +1658,8 @@
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>How to apply for an OEC online, as the website is down.</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2141,16 +1674,8 @@
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>If deported, can I still work in other countries?</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2165,16 +1690,8 @@
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Reduced my salary for electricity, is that correct?</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2189,16 +1706,8 @@
       </c>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>Can assistance be requested from OWWA for a legal battle?</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2213,16 +1722,8 @@
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>I was accused of theft without evidence, can I file a lawsuit?</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2237,16 +1738,8 @@
       </c>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>I wish to resign but has a bond.</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2261,16 +1754,8 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>I am being forced to sign a document that I do not understand.</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2285,16 +1770,8 @@
       </c>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Is it true that placement fees are prohibited for domestic helpers?</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2309,16 +1786,8 @@
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>How should I proceed if my visa has expired while waiting for the new contract?</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2333,16 +1802,8 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>I am physically abused by my employer, where should I report?</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2357,16 +1818,8 @@
       </c>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Please explain the One Month Notice rule.</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2381,16 +1834,8 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Can an employee work part-time during their day off to earn extra?</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2405,16 +1850,8 @@
       </c>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Cancelled my visa without informing me, is that legal?</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2429,16 +1866,8 @@
       </c>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>What should be done, I do not want to be given a release letter?</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2453,16 +1882,8 @@
       </c>
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Can an individual file an anonymous complaint with DOLE?</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2477,16 +1898,8 @@
       </c>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>The alleged delayed salary constitutes grounds for termination.</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2501,16 +1914,8 @@
       </c>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>What is the coverage of the insurance in case of an accident at work?</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2525,16 +1930,8 @@
       </c>
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Is the use of mobile phones during working hours prohibited?</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2549,16 +1946,8 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>The employer expelled the employee from the house last night.</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2573,16 +1962,8 @@
       </c>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>Is the 24-hour monitoring in my room via CCTV legal?</t>
-        </is>
-      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2597,16 +1978,8 @@
       </c>
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>What is the procedure for direct hiring through an agency?</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2621,16 +1994,8 @@
       </c>
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>How to claim OWWA benefits if I am a member?</t>
-        </is>
-      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2645,16 +2010,8 @@
       </c>
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>What are the requirements for Balik Manggagawa?</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2669,16 +2026,8 @@
       </c>
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>I am awaiting departure orders, how will I know?</t>
-        </is>
-      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2693,16 +2042,8 @@
       </c>
       <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Can the spouse file an adultery case against me even if I am abroad?</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2717,16 +2058,8 @@
       </c>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>Where can an abusive agency be reported?</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2741,16 +2074,8 @@
       </c>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>If I am terminated, will they return my ticket?</t>
-        </is>
-      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2765,16 +2090,8 @@
       </c>
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Is the contract valid without a POEA signature?</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2789,16 +2106,8 @@
       </c>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>I am being detained by immigration, what should be done?</t>
-        </is>
-      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2813,16 +2122,8 @@
       </c>
       <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Tagalog</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Renewal of passport pages is required at the consulate?</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2837,16 +2138,8 @@
       </c>
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>I did not receive MPF payments from my employer. Can a report be filed?</t>
-        </is>
-      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2861,16 +2154,8 @@
       </c>
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>The employer's failure to provide notice period prior to termination is unlawful.</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2885,16 +2170,8 @@
       </c>
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>I have worked for five years, should I be entitled to long service leave?</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2909,16 +2186,8 @@
       </c>
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>The visa has expired for two days. Will the individual be deported?</t>
-        </is>
-      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2933,16 +2202,8 @@
       </c>
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>I am alleged to have damaged property, but I have not done so.</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2957,16 +2218,8 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>I was not given a ticket back to the Philippines. Where can I file a complaint?</t>
-        </is>
-      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2981,16 +2234,8 @@
       </c>
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>Terminate contract, require how much notice?</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3005,16 +2250,8 @@
       </c>
       <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>If an employee works a part-time job during their vacation period, would that be illegal?</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3029,16 +2266,8 @@
       </c>
       <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>The employer has taken the passport and refuses to return it.</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3053,16 +2282,8 @@
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>What is the contact number of the Labour Department? I would like to inquire about workers' compensation.</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3077,16 +2298,8 @@
       </c>
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>They do not give me a holiday, saying they need to pay me money, is that allowed?</t>
-        </is>
-      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3101,16 +2314,8 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>I have not completed the contract, may I switch to a new employer?</t>
-        </is>
-      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3125,16 +2330,8 @@
       </c>
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr"/>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>The employer did not provide insurance, what should be done when I became ill?</t>
-        </is>
-      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3149,16 +2346,8 @@
       </c>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr"/>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>I was accused of stealing and was reported to the police, but I did not do it.</t>
-        </is>
-      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3173,16 +2362,8 @@
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Do I have to live at the employer's house? Can I go out and live elsewhere?</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3197,16 +2378,8 @@
       </c>
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Chinese</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>How much money must be paid if an employee resigns during the probation period?</t>
-        </is>
-      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3221,16 +2394,8 @@
       </c>
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>I was beaten by my employer, do I have the right to sue him?</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3245,16 +2410,8 @@
       </c>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>They do not provide me with enough food to eat, does this constitute abuse?</t>
-        </is>
-      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3269,16 +2426,8 @@
       </c>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Can they fire me if I am pregnant?</t>
-        </is>
-      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3293,16 +2442,8 @@
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>The intermediary company collected a large amount of money from me. Is this illegal?</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3317,16 +2458,8 @@
       </c>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>Can the person refuse to go to the second location?</t>
-        </is>
-      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3341,16 +2474,8 @@
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>What are the legal implications of debt on visa application?</t>
-        </is>
-      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3365,16 +2490,8 @@
       </c>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>Does the contract remain valid after the employer's death?</t>
-        </is>
-      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3389,16 +2506,8 @@
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>How is the mandatory provident fund contribution calculated?</t>
-        </is>
-      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3413,16 +2522,8 @@
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>I was not given notice of the termination, can I pursue legal action?</t>
-        </is>
-      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3437,16 +2538,8 @@
       </c>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr"/>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Can the contract be canceled after signing?</t>
-        </is>
-      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3461,16 +2554,8 @@
       </c>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>They installed CCTV in the restroom, I am very scared.</t>
-        </is>
-      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3485,16 +2570,8 @@
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr"/>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>I am required to work 20 hours per day, which is not feasible, can I report to the labor department?</t>
-        </is>
-      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3509,16 +2586,8 @@
       </c>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr"/>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>I have not received the last installment of food.</t>
-        </is>
-      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3533,16 +2602,8 @@
       </c>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr"/>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Chinese</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>What is the legal recourse for wrongful termination?</t>
-        </is>
-      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3557,16 +2618,8 @@
       </c>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr"/>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>They do not believe in religion as I do, nor do they go to church with me.</t>
-        </is>
-      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3581,16 +2634,8 @@
       </c>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr"/>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>Departure is required when the visa is denied.</t>
-        </is>
-      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3605,16 +2650,8 @@
       </c>
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr"/>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>I have lost a contract, where to obtain a replacement?</t>
-        </is>
-      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3629,16 +2666,8 @@
       </c>
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr"/>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>Can an employee refuse dangerous work requested by the employer?</t>
-        </is>
-      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3653,16 +2682,8 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr"/>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>The subjects do not communicate with their family members via telephone.</t>
-        </is>
-      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3677,16 +2698,8 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>What is the procedure for renewing a contract?</t>
-        </is>
-      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3701,16 +2714,8 @@
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>What is the legal requirement regarding vacation leave?</t>
-        </is>
-      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3725,16 +2730,8 @@
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>The employer refuses to issue a resignation letter to me.</t>
-        </is>
-      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3749,16 +2746,8 @@
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>Go to the embassy first due to labor disputes.</t>
-        </is>
-      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3773,16 +2762,8 @@
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr"/>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>I was prevented from reading my letter.</t>
-        </is>
-      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3797,16 +2778,8 @@
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr"/>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>Is the injury considered a work-related injury?</t>
-        </is>
-      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3821,16 +2794,8 @@
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr"/>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>Is it illegal for the employer to not provide rest days?</t>
-        </is>
-      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3845,16 +2810,8 @@
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>Can a relative stay overnight?</t>
-        </is>
-      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3869,16 +2826,8 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>Help me check the shop, okay?</t>
-        </is>
-      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3893,16 +2842,8 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>Who will pay for the ticket if the contract is terminated early?</t>
-        </is>
-      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3917,16 +2858,8 @@
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr"/>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Cantonese</t>
-        </is>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>Am I required to follow my boss to immigrate?</t>
-        </is>
-      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3992,6 +2925,294 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr"/>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>我啱啱發現有咗BB，老細知道之後即刻話要炒我，香港法例係咪容許咁樣？</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>其實我做得好唔開心想自己斷約，但係我無錢賠一個月糧，可唔可以即刻走？</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>呢幾個月老細都係遲出糧，有時拖成十幾日，我投訴佢就話無錢，我可唔可以當佢自動解僱我？</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>每個月出糧佢都淨係俾三千幾蚊我，話扣起咗啲做中介費，但我未簽過任何同意書。</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>合約寫明包食宿，但每個月都冇比膳食津貼，又要我用自己人工買餸自己煮，算唔算犯法？</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>佢哋安排我同個十歲嘅男仔同埋老爺一間房訓，我覺得好唔舒服，勞工處有冇規定住宿環境？</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>我發高燒入咗醫院，僱主話醫藥費太貴唔肯幫我比，仲話要扣我人工當醫藥費。</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>每日由朝早六點做到半夜一點，完全無私人時間休息，我有冇權利要求固定休息時間？</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>僱主逼我簽一份『自願離職』信，話唔簽就報警屈我偷嘢，我好驚，點算好？</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>做咗三個月，僱主話我做嘢太慢終止合約，佢係咪需要負責我返去嘅機票？</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>僱主突然話聽日唔洗我返工，又唔補一個月代通知金比我，我依家可以點做？</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>我不小心整爛咗個微波爐，老細今個月扣咗我二千蚊人工，佢係咪可以扣咁多？</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>佢話我上星期表現唔好，所以今個月要扣減五百蚊人工當懲罰，勞工法例有冇話唔得？</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr"/>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>我抹緊窗嗰陣跌親隻手，但僱主冇幫我買勞保，依家唔肯負責我嘅物理治療費用，點算？</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>老細成日用粗口鬧我，有時仲會掟嘢，我覺得人身安全受威脅，佢咁做算唔算違反僱傭合約？</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>老細叫我星期日放假都要留喺屋企照顧小朋友，話補返一百蚊比我，我可唔可以拒絕？</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>婆婆（受照顧者）過身，佢個仔話合約即刻完，要我聽日就買機票返菲律賓，咁我啲遣散費點計？</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr"/>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>我平時除咗做家務，老細仲日日叫我落去佢間茶餐廳幫手洗碗，咁樣係咪做緊黑工？</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Cantonese</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>